<commit_message>
Update data tables and main menu UI
</commit_message>
<xml_diff>
--- a/Excel/BlueprintConfig.xlsx
+++ b/Excel/BlueprintConfig.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -477,20 +477,20 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>blueprint_maze_energy</t>
+          <t>blueprint_maze_energy_small</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>迷宫节能图纸</t>
+          <t>轻装探索图纸</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>buff_maze_energy</t>
+          <t>buff_maze_energy_small</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -502,55 +502,205 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>blueprint_craft_double</t>
+          <t>blueprint_maze_energy</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>制作灵感图纸</t>
+          <t>节能步伐图纸</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>150</v>
+        <v>260</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>buff_craft_double</t>
+          <t>buff_maze_energy</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[clear_forest_maze]</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>blueprint_shop_speed</t>
+          <t>blueprint_maze_energy_large</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>店铺招牌图纸</t>
+          <t>迷宫指南针图纸</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>200</v>
+        <v>520</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>buff_shop_speed</t>
+          <t>buff_maze_energy_large</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[clear_depth_maze]</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
+        <is>
+          <t>blueprint_craft_double_small</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>灵感火花图纸</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>140</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>buff_craft_double_small</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>blueprint_craft_double</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>料理直觉图纸</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>300</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>buff_craft_double</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>[food_carrot_soup]</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>blueprint_craft_double_large</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>大师备餐术图纸</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>620</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>buff_craft_double_large</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>[food_maze_bento]</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>blueprint_shop_speed_small</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>热情招呼图纸</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>160</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>buff_shop_speed_small</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>blueprint_shop_speed</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>醒目招牌图纸</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>340</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>buff_shop_speed</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>[food_mushroom_skewer]</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>blueprint_shop_speed_large</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>黄金营业时段图纸</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>680</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>buff_shop_speed_large</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>[food_feast_platter]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>END</t>
         </is>

</xml_diff>